<commit_message>
Publish source only and exclude Electron build artifacts
</commit_message>
<xml_diff>
--- a/src/assets/templates/10-ROGNONI-Rilevazione_estratti_template.xlsx
+++ b/src/assets/templates/10-ROGNONI-Rilevazione_estratti_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rt080\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://beyondoc-my.sharepoint.com/personal/thomas_rognoni_beyondoc_com/Documents/Desktop/Angular/monthly-report-app/src/assets/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4ECB242-BBDC-4905-AA50-97107C7B4E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{B4ECB242-BBDC-4905-AA50-97107C7B4E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88F96528-4E90-4DC8-93E9-C3F1C38B7FCC}"/>
   <bookViews>
-    <workbookView xWindow="-4116" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{A65CC0B0-33FF-4917-A142-09106219D7C1}"/>
+    <workbookView xWindow="-3912" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{A65CC0B0-33FF-4917-A142-09106219D7C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -999,7 +999,7 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>1830450</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>178371</xdr:rowOff>
+      <xdr:rowOff>173291</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1979,7 +1979,7 @@
       <c r="G8" s="5"/>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="2:8" ht="9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="10"/>
       <c r="C9" s="61"/>
       <c r="D9" s="89"/>
@@ -5811,19 +5811,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1f0977cb-d2f3-45c6-84d8-726f35a87576" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e" xsi:nil="true"/>
-    <LUGAMM xmlns="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e">true</LUGAMM>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007DA27F5BB0A1F44CB2271C3F58AABC4A" ma:contentTypeVersion="16" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="6c38615e733aadaab643e8f4522f5d8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e" xmlns:ns3="1f0977cb-d2f3-45c6-84d8-726f35a87576" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4078b8ab279635d84e8c1adaf3d54276" ns2:_="" ns3:_="">
     <xsd:import namespace="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e"/>
@@ -6064,6 +6051,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1f0977cb-d2f3-45c6-84d8-726f35a87576" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e" xsi:nil="true"/>
+    <LUGAMM xmlns="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e">true</LUGAMM>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E35DA4B-C97A-4E5A-819C-E333005729F9}">
   <ds:schemaRefs>
@@ -6073,17 +6073,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F747A2-FC3D-47C9-9015-4E8B364ECFA3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e"/>
-    <ds:schemaRef ds:uri="1f0977cb-d2f3-45c6-84d8-726f35a87576"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05E156EB-A677-4784-8A77-9C20301CB2A4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6100,4 +6089,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F747A2-FC3D-47C9-9015-4E8B364ECFA3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="31a33ae0-9583-4d24-8d2a-dd0d1d8b938e"/>
+    <ds:schemaRef ds:uri="1f0977cb-d2f3-45c6-84d8-726f35a87576"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>